<commit_message>
New Excel template file
</commit_message>
<xml_diff>
--- a/resume_template.xlsx
+++ b/resume_template.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="83">
   <si>
     <t>date</t>
   </si>
@@ -279,6 +279,15 @@
   </si>
   <si>
     <t>2025-10-16 10:37:22</t>
+  </si>
+  <si>
+    <t>2025-10-17 11:03:04</t>
+  </si>
+  <si>
+    <t>2025-10-17 11:03:05</t>
+  </si>
+  <si>
+    <t>2025-10-17 11:03:06</t>
   </si>
 </sst>
 </file>
@@ -1087,7 +1096,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D143"/>
+  <dimension ref="A1:D149"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="24.140625"/>
@@ -3086,15 +3095,99 @@
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B143" s="1">
+        <v>45946</v>
+      </c>
+      <c r="C143" t="s">
+        <v>17</v>
+      </c>
+      <c r="D143">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A144" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B144" s="1">
+        <v>45946</v>
+      </c>
+      <c r="C144" t="s">
+        <v>18</v>
+      </c>
+      <c r="D144">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A145" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B145" s="1">
+        <v>45946</v>
+      </c>
+      <c r="C145" t="s">
+        <v>19</v>
+      </c>
+      <c r="D145">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A146" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B146" s="1">
+        <v>45946</v>
+      </c>
+      <c r="C146" t="s">
+        <v>20</v>
+      </c>
+      <c r="D146">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A147" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B147" s="1">
+        <v>45946</v>
+      </c>
+      <c r="C147" t="s">
+        <v>11</v>
+      </c>
+      <c r="D147">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A148" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B148" s="1">
+        <v>45946</v>
+      </c>
+      <c r="C148" t="s">
+        <v>12</v>
+      </c>
+      <c r="D148">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A149" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B143" s="1" t="s">
+      <c r="B149" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C143" t="s">
+      <c r="C149" t="s">
         <v>6</v>
       </c>
-      <c r="D143" t="s">
+      <c r="D149" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>